<commit_message>
Normalize nearby-card titles to official neighborhood names
The audit now also rewrites each 'Nearby Neighborhood N - Title' to the
referenced row's Neighborhood Name (18 cells: missing 'The ' prefixes plus
one missing 'Club' suffix). The workbook gains a Title Changes sheet and
the import CSV carries all three fixes: 388 descriptions, 18 titles,
22 links.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0151vzeDTEiwBUT4icARckom
</commit_message>
<xml_diff>
--- a/audit/Nearby-Neighborhood-Descriptions-Update.xlsx
+++ b/audit/Nearby-Neighborhood-Descriptions-Update.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Paste into Wix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Changed Cells" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Link Issues" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Title Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Link Issues" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -644,9 +645,9 @@
           <t>Sea Gate Club is a Gulf-front condominium tower of 90 residences on Longboat Key, set on the beach with golf across the street and the island's main shopping plaza steps away. Residents enjoy a Gulf-side heated pool and spa, tennis, a fitness center, a social room, and on-site management. Most homes are two-bedroom split plans with floor-to-ceiling windows and balconies framing Gulf and bay views.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Islander Club</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1018,9 +1019,9 @@
           <t>The Privateer is a Gulf-front condominium community of two high-rise towers on the south end of Longboat Key. Residents here enjoy a Gulf-front pool, tennis courts, pickleball, fitness center, clubhouse and more.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Water Club</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1330,9 +1331,9 @@
           <t>The Players Club is an exclusive luxury condo community right on the water.  It has 134 residences in 4 mid-rise buildings. Amenities are plentiful and include a private beach, a large heated pool and spa, four Har-Tru tennis courts, a putting green, and a clubhouse with a fitness center.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Water Club</t>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1674,9 +1675,9 @@
           <t>3ccb68d1-2269-4a6d-b4ac-5175a8f82fc1</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Bayport Beach &amp; Tennis</t>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Bayport Beach &amp; Tennis Club</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1892,9 +1893,9 @@
           <t>Villa di Lancia is a gated beachside community of 38 residences in two Mediterranean-style buildings on the south end of Longboat Key. Five acres of grounds hold a heated pool and hot tub, two Har-Tru tennis/pickleball courts, and a clubhouse with a fitness room and sauna. With homes running from about 2,400 to nearly 5,000 square feet, it suits buyers who want house-sized living right on the sand.</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Islander Club</t>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1954,9 +1955,9 @@
           <t>Sage Longboat Key is one of the newest boutique Gulf-front condominiums on Longboat Key. There are just 16 residences here. Each home spans the full width of the building, with views of both the Gulf and Sarasota Bay. Wellness anchors the design, from air and water filtration to a beautiful pool, spa, fitness center, and yoga studio.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Castillian</t>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -2142,9 +2143,9 @@
           <t>56c00258-e6c1-4aa2-aaa4-9ca4c15dad5f</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Water Club</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2204,9 +2205,9 @@
           <t>La Playa is an intimate Gulf-front community of just 21 residences set directly on a private beach in the heart of Longboat Key. Amenities include a heated pool and beachfront grills just off the sand. As one of the few communities on the island that permits short-term rentals, it draws owners who want a beach residence that can also generate rental income.</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Castillian</t>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2370,9 +2371,9 @@
           <t>En Provence is a 21-residence ultra-luxury community on six Gulf-front acres near the south end of Longboat Key, with estate-scale floor plans of 3,400 to over 6,000 square feet, private elevators, and enclosed garages. Amenities include a heated beachfront pool and spa, fitness center, clubhouse with catering kitchen, concierge, and 24-hour guard-gated security.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Islander Club</t>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2474,9 +2475,9 @@
           <t>Veinte takes its name from the Spanish word for twenty, and that's exactly how many residences share this Gulf-front mid-rise on Longboat Key. Homes here offer direct Gulf views, and residents share a heated pool facing the water, a tennis/pickleball court, and a private beach. Sitting directly across from Publix and the town's public tennis center, it's a strong fit for buyers who want Gulf-front living with daily errands minutes from the door.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Beachcomber</t>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2766,9 +2767,9 @@
           <t>6dbf2382-6ba6-4d57-ace5-7ad0087248f3</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Beachcomber</t>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -4086,9 +4087,9 @@
           <t>Islands West is a Gulf-front high-rise featuring private beach access, a heated beachfront pool, fitness center, sauna, tennis, and social spaces. It offers a traditional beachfront tower lifestyle with strong core amenities.</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Islander Club</t>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
@@ -4118,9 +4119,9 @@
           <t>a6ddaacc-14e5-4041-a123-ef4ec9bd5640</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Castillian</t>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -4284,9 +4285,9 @@
           <t>Beachplace is a large resort-style beachfront community with several resort-style amenities. These include private beach access, a community pool, clubhouse, fitness center, and tennis/pickleball.</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>Water Club</t>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -4502,9 +4503,9 @@
           <t>Longboat Harbour is likely the ultimate Bay-side boating community on Longboat Key. It consists of around 300 condominiums with berths for more than 50 boats and accommodates vessels up to 34 feet. Amenities include tennis/pickleball courts, a fitness center, a large bayfront clubhouse, active social calendar and more.</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Castillian</t>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
@@ -4846,9 +4847,9 @@
           <t>c92a6bc1-a2f7-4df5-ae83-5e46e18cda2f</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Beachcomber</t>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -5688,9 +5689,9 @@
           <t>Casa Del Mar is a Gulf-front condominium community offering direct beach access, a beachfront pool, and tennis and pickleball courts. It's well suited for buyers wanting a casual, resort-style setting with strong vacation, seasonal, and rental income appeal.</t>
         </is>
       </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>Castillian</t>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -5968,9 +5969,9 @@
           <t>Sunset Beach is a gated community of 3 mid-rise buildings directly on the Gulf, toward the south end of Longboat Key. With just over 60 condominiums, residents enjoy a private beach, heated pool, club room, kayak storage, and under-building parking. Its location is also next to the golf course and - true to its name - the sunsets are spectacular.</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>Islander Club</t>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="J106" s="3" t="inlineStr">
@@ -6270,7 +6271,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Islander Club</t>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -7134,7 +7135,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Water Club</t>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -7806,7 +7807,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Water Club</t>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -8606,7 +8607,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Bayport Beach &amp; Tennis</t>
+          <t>Bayport Beach &amp; Tennis Club</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -9150,7 +9151,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Islander Club</t>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -9310,7 +9311,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Castillian</t>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -9726,7 +9727,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Water Club</t>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -9854,7 +9855,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Castillian</t>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -10238,7 +10239,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Islander Club</t>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -10462,7 +10463,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Beachcomber</t>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -11134,7 +11135,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Beachcomber</t>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -14110,7 +14111,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Islander Club</t>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -14174,7 +14175,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Castillian</t>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -14526,7 +14527,7 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Water Club</t>
+          <t>The Water Club</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -15006,7 +15007,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Castillian</t>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -15838,7 +15839,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Beachcomber</t>
+          <t>The Beachcomber</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -17758,7 +17759,7 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>Castillian</t>
+          <t>The Castillian</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
@@ -18430,7 +18431,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>Islander Club</t>
+          <t>The Islander Club</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -18455,6 +18456,444 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Neighborhood (row)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Current Title</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Official Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Vizcaya</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Islander Club</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Beachplace</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Water Club</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>The Residences at The St. Regis</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Water Club</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Beach Harbor Club</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Bayport Beach &amp; Tennis</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Bayport Beach &amp; Tennis Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Aria</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Islander Club</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Casa Del Mar</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Castillian</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Players Club</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Water Club</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Arbomar</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Castillian</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Villa di Lancia</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Islander Club</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Islands West</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Beachcomber</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Neptune</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Beachcomber</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Sea Gate Club</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Islander Club</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Longboat Harbour</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Castillian</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Promenade</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Water Club</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>The Water Club</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>La Firenza</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Castillian</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Veinte</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Beachcomber</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>The Beachcomber</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>The Grande at Longboat Key</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Castillian</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>The Castillian</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Fairway Bay (Bay Isles)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Islander Club</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>The Islander Club</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>